<commit_message>
fix: certificate coordinates and pdf improvements
</commit_message>
<xml_diff>
--- a/backend/data/users.xlsx
+++ b/backend/data/users.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="138" uniqueCount="86">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="152" uniqueCount="95">
   <si>
     <t>الاسم بالعربية</t>
   </si>
@@ -269,6 +269,33 @@
   </si>
   <si>
     <t>EVC-9903CCDC</t>
+  </si>
+  <si>
+    <t>سامر</t>
+  </si>
+  <si>
+    <t>Samer</t>
+  </si>
+  <si>
+    <t>samer@gmail.com</t>
+  </si>
+  <si>
+    <t>00000000000</t>
+  </si>
+  <si>
+    <t>EVC-CA088494</t>
+  </si>
+  <si>
+    <t>ماجستير</t>
+  </si>
+  <si>
+    <t>sssssssssssssss</t>
+  </si>
+  <si>
+    <t>sssssssssssss</t>
+  </si>
+  <si>
+    <t>٢٣‏/٤‏/٢٠٢٦</t>
   </si>
 </sst>
 </file>
@@ -704,7 +731,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:N20"/>
+  <dimension ref="A1:N21"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="2" width="25" customWidth="1"/>
@@ -1303,6 +1330,50 @@
         <v>61</v>
       </c>
     </row>
+    <row r="21" ht="20" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A21" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="B21" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="C21" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="D21" s="4" t="s">
+        <v>89</v>
+      </c>
+      <c r="E21" s="4" t="s">
+        <v>90</v>
+      </c>
+      <c r="F21" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="G21" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="H21" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="I21" s="4" t="s">
+        <v>91</v>
+      </c>
+      <c r="J21" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="K21" s="4" t="s">
+        <v>93</v>
+      </c>
+      <c r="L21" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="M21" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="N21" s="4" t="s">
+        <v>94</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>

</xml_diff>